<commit_message>
masters: regenereret fra plan.json
</commit_message>
<xml_diff>
--- a/data/Fast_as_Fifty_Masterplan_2026.xlsx
+++ b/data/Fast_as_Fifty_Masterplan_2026.xlsx
@@ -487,14 +487,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="62" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="58" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -721,6 +722,11 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
+          <t>Tilmeldt</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
           <t>Note</t>
         </is>
       </c>
@@ -736,9 +742,18 @@
           <t>2026-08-29</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr"/>
-      <c r="D16" s="4" t="inlineStr"/>
-      <c r="E16" s="5" t="inlineStr"/>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>2000m</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr"/>
+      <c r="F16" s="5" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -751,14 +766,23 @@
           <t>2026-09-05</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr"/>
-      <c r="D17" s="4" t="inlineStr"/>
-      <c r="E17" s="5" t="inlineStr"/>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>42.2km</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr"/>
+      <c r="F17" s="5" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Stelvio Gran Fondo</t>
+          <t>Santini Stelvio Gran Fondo (lang rute)</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
@@ -771,10 +795,19 @@
           <t>B</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr"/>
-      <c r="E18" s="5" t="inlineStr">
-        <is>
-          <t>Hyggetur med Eva + form-check.</t>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>130km / 4500hm</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Ja (2026-07-16)</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>B-løb. TILMELDT 16/7-2026 (med Eva). Hyggeløb + form-check mod TdS.</t>
         </is>
       </c>
     </row>
@@ -796,12 +829,17 @@
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>242 km / 8.848 hm</t>
-        </is>
-      </c>
-      <c r="E19" s="5" t="inlineStr">
-        <is>
-          <t>Start 02:30. Sæsonens hovedmål.</t>
+          <t>242km / 8848hm</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>Nej</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>A-løb. IKKE TILMELDT — 2027 åbner først ca. sep-26. Tjek 20/9. Cutoff 20:30 Croix-de-Cœur. Start 02:30 (18 t margin).</t>
         </is>
       </c>
     </row>
@@ -2927,7 +2965,7 @@
       </c>
       <c r="J43" s="5" t="inlineStr">
         <is>
-          <t>STELVIO GRAN FONDO søn 6/6 — B-løb. Hyggetur med Eva + form-check.</t>
+          <t>LA STELVIO SANTINI (Santini Stelvio Gran Fondo, lang rute) søn 6/6 — 130 km / 4.500 hm. B-løb, tilmeldt 16/7-2026 sammen med Eva. Form-check mod TdS: kør den som hårdt træningspas, ikke som A-løb.</t>
         </is>
       </c>
     </row>
@@ -5948,8 +5986,12 @@
       <c r="F5" s="4" t="n">
         <v>290</v>
       </c>
-      <c r="G5" s="4" t="n"/>
-      <c r="H5" s="11" t="n"/>
+      <c r="G5" s="4" t="n">
+        <v>284</v>
+      </c>
+      <c r="H5" s="11" t="n">
+        <v>-6</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
@@ -5974,8 +6016,12 @@
       <c r="F6" s="4" t="n">
         <v>340</v>
       </c>
-      <c r="G6" s="4" t="n"/>
-      <c r="H6" s="11" t="n"/>
+      <c r="G6" s="4" t="n">
+        <v>451</v>
+      </c>
+      <c r="H6" s="11" t="n">
+        <v>111</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
@@ -6000,8 +6046,12 @@
       <c r="F7" s="4" t="n">
         <v>370</v>
       </c>
-      <c r="G7" s="4" t="n"/>
-      <c r="H7" s="11" t="n"/>
+      <c r="G7" s="4" t="n">
+        <v>386</v>
+      </c>
+      <c r="H7" s="11" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
@@ -6026,8 +6076,12 @@
       <c r="F8" s="4" t="n">
         <v>180</v>
       </c>
-      <c r="G8" s="4" t="n"/>
-      <c r="H8" s="11" t="n"/>
+      <c r="G8" s="4" t="n">
+        <v>367</v>
+      </c>
+      <c r="H8" s="11" t="n">
+        <v>187</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
@@ -6052,8 +6106,12 @@
       <c r="F9" s="4" t="n">
         <v>385</v>
       </c>
-      <c r="G9" s="4" t="n"/>
-      <c r="H9" s="11" t="n"/>
+      <c r="G9" s="4" t="n">
+        <v>558</v>
+      </c>
+      <c r="H9" s="11" t="n">
+        <v>173</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
@@ -6078,8 +6136,12 @@
       <c r="F10" s="4" t="n">
         <v>300</v>
       </c>
-      <c r="G10" s="4" t="n"/>
-      <c r="H10" s="11" t="n"/>
+      <c r="G10" s="4" t="n">
+        <v>267</v>
+      </c>
+      <c r="H10" s="11" t="n">
+        <v>-33</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
@@ -6104,8 +6166,12 @@
       <c r="F11" s="4" t="n">
         <v>430</v>
       </c>
-      <c r="G11" s="4" t="n"/>
-      <c r="H11" s="11" t="n"/>
+      <c r="G11" s="4" t="n">
+        <v>455</v>
+      </c>
+      <c r="H11" s="11" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
@@ -6130,8 +6196,12 @@
       <c r="F12" s="4" t="n">
         <v>480</v>
       </c>
-      <c r="G12" s="4" t="n"/>
-      <c r="H12" s="11" t="n"/>
+      <c r="G12" s="4" t="n">
+        <v>417</v>
+      </c>
+      <c r="H12" s="11" t="n">
+        <v>-63</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
@@ -6156,8 +6226,12 @@
       <c r="F13" s="4" t="n">
         <v>270</v>
       </c>
-      <c r="G13" s="4" t="n"/>
-      <c r="H13" s="11" t="n"/>
+      <c r="G13" s="4" t="n">
+        <v>363</v>
+      </c>
+      <c r="H13" s="11" t="n">
+        <v>93</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
@@ -6183,10 +6257,10 @@
         <v>420</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>199</v>
+        <v>234</v>
       </c>
       <c r="H14" s="11" t="n">
-        <v>-221</v>
+        <v>-186</v>
       </c>
     </row>
     <row r="15">

</xml_diff>